<commit_message>
using ocr and pymupdf
</commit_message>
<xml_diff>
--- a/data/pdfs/excel stream karnivel.xlsx
+++ b/data/pdfs/excel stream karnivel.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\projects\whatsapp integration\data\pdfs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A39E9F5-13AF-4B6C-963C-14DB2BD0908A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE14A5AF-74BD-41FD-82DD-646F786AE123}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2550" yWindow="2550" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -352,7 +352,100 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="5">
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="20"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="20"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="20"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="20"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="20"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="23" formatCode="h:mm\ AM/PM"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -363,6 +456,19 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{87FE4F3F-6FA1-43DD-83A3-B40CD7A5EF37}" name="Table1" displayName="Table1" ref="A1:D141" totalsRowShown="0" headerRowDxfId="0">
+  <autoFilter ref="A1:D141" xr:uid="{87FE4F3F-6FA1-43DD-83A3-B40CD7A5EF37}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{6349D0B5-6BE8-4DCC-9A9B-7058AFD84141}" name="Time" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{F3BA06C1-BEF3-4903-B481-9F4710EF04A2}" name="Item" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{72406AFF-7F5C-49C1-9DC7-5A8E2C09FCF7}" name="Category" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{2ED12FBF-E30B-461E-891A-0DAE3A1BE15A}" name="Date" dataDxfId="1"/>
+  </tableColumns>
+  <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -10572,5 +10678,8 @@
   <printOptions horizontalCentered="1" gridLines="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup fitToHeight="0" pageOrder="overThenDown" orientation="landscape" cellComments="atEnd"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>